<commit_message>
Fix draft privacy, admin workflow and Excel export formatting
</commit_message>
<xml_diff>
--- a/docs/虚构数据_2026-09_v1.xlsx
+++ b/docs/虚构数据_2026-09_v1.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="24">
   <si>
     <t>姓名</t>
   </si>
@@ -45,18 +45,18 @@
     <t>0000001001</t>
   </si>
   <si>
+    <t>活动文案整理</t>
+  </si>
+  <si>
+    <t>真实工作8小时（虚构示例）</t>
+  </si>
+  <si>
     <t>物料费用折算</t>
   </si>
   <si>
     <t>物料费30元÷25=1.2小时</t>
   </si>
   <si>
-    <t>活动文案整理</t>
-  </si>
-  <si>
-    <t>真实工作8小时（虚构示例）</t>
-  </si>
-  <si>
     <t>交通费用折算</t>
   </si>
   <si>
@@ -72,10 +72,13 @@
     <t>统计月份：2026-09 ｜ 导出时间：2026/9/30 18:00:00（北京时间） ｜ 版本：v1</t>
   </si>
   <si>
-    <t>已通过3条，11.2004小时，280.01元；仅合计行E列展示金额，明细E列为备注。</t>
-  </si>
-  <si>
-    <t>费用已折算包含在工时内，不重复加款。按组内个人合计舍入到分；本组排除0条。</t>
+    <t>已通过3条，11.2004小时，280.01元；合计行E列展示金额，明细E列为备注。</t>
+  </si>
+  <si>
+    <t>费用已包含在工时内，不重复加款。正式记录排除0条；另有未提交草稿0条（仅数量）。</t>
+  </si>
+  <si>
+    <t>金额按组内个人合计舍入到分；长文本可能续行，工时仅在该记录首行计入。</t>
   </si>
   <si>
     <t>已通过、已导出仅表示审核与整理进度，不代表款项已到账。</t>
@@ -97,10 +100,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.####"/>
     <numFmt numFmtId="165" formatCode="&quot;金额：&quot;0.00&quot; 元&quot;"/>
-    <numFmt numFmtId="166" formatCode="0.####&quot; 小时&quot;"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -133,7 +135,7 @@
       <name val="Microsoft YaHei"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -143,6 +145,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF7F6F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF3F2EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE6E5DF"/>
       </patternFill>
     </fill>
   </fills>
@@ -158,33 +170,50 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -528,7 +557,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -538,7 +567,7 @@
     <col min="5" max="5" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -566,7 +595,7 @@
         <v>7</v>
       </c>
       <c r="D2" s="6">
-        <v>1.2</v>
+        <v>8</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>8</v>
@@ -583,7 +612,7 @@
         <v>9</v>
       </c>
       <c r="D3" s="6">
-        <v>8</v>
+        <v>1.2</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>10</v>
@@ -606,7 +635,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>5</v>
       </c>
@@ -625,63 +654,73 @@
         <v>280.01</v>
       </c>
     </row>
-    <row r="6" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
+    <row r="6" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="12">
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="14">
         <f>SUM(D5)</f>
         <v>11.2004</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="11">
+      <c r="E6" s="15">
         <f>SUM(E5)</f>
         <v>280.01</v>
       </c>
     </row>
-    <row r="8" ht="32" customHeight="1" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+    <row r="8" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-    </row>
-    <row r="9" ht="32" customHeight="1" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="14" t="s">
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+    </row>
+    <row r="9" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-    </row>
-    <row r="10" ht="32" customHeight="1" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="14" t="s">
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+    </row>
+    <row r="10" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-    </row>
-    <row r="11" ht="32" customHeight="1" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+    </row>
+    <row r="11" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+    </row>
+    <row r="12" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A8:E8"/>
     <mergeCell ref="A9:E9"/>
     <mergeCell ref="A10:E10"/>
     <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A12:E12"/>
   </mergeCells>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
@@ -692,7 +731,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -702,7 +741,7 @@
     <col min="5" max="5" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -730,7 +769,7 @@
         <v>9</v>
       </c>
       <c r="D2" s="6">
-        <v>8</v>
+        <v>1.2</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>10</v>
@@ -744,13 +783,13 @@
         <v>6</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D3" s="6">
-        <v>2.0004</v>
+        <v>8</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" ht="25" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -761,16 +800,16 @@
         <v>6</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D4" s="6">
-        <v>1.2</v>
+        <v>2.0004</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>5</v>
       </c>
@@ -789,63 +828,73 @@
         <v>280.01</v>
       </c>
     </row>
-    <row r="6" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
+    <row r="6" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="12">
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="14">
         <f>SUM(D5)</f>
         <v>11.2004</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="11">
+      <c r="E6" s="15">
         <f>SUM(E5)</f>
         <v>280.01</v>
       </c>
     </row>
-    <row r="8" ht="32" customHeight="1" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+    <row r="8" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-    </row>
-    <row r="9" ht="32" customHeight="1" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="14" t="s">
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+    </row>
+    <row r="9" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-    </row>
-    <row r="10" ht="32" customHeight="1" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="14" t="s">
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+    </row>
+    <row r="10" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-    </row>
-    <row r="11" ht="32" customHeight="1" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+    </row>
+    <row r="11" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+    </row>
+    <row r="12" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A8:E8"/>
     <mergeCell ref="A9:E9"/>
     <mergeCell ref="A10:E10"/>
     <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A12:E12"/>
   </mergeCells>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
@@ -856,7 +905,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -866,7 +915,7 @@
     <col min="5" max="5" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -885,16 +934,16 @@
     </row>
     <row r="2" ht="25" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>7</v>
       </c>
       <c r="D2" s="6">
-        <v>1.2</v>
+        <v>8</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>8</v>
@@ -902,44 +951,44 @@
     </row>
     <row r="3" ht="25" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D3" s="6">
-        <v>8</v>
+        <v>2.0004</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" ht="25" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="6">
+        <v>1.2</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="6">
-        <v>2.0004</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
-        <v>19</v>
-      </c>
       <c r="B5" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>13</v>
@@ -953,63 +1002,73 @@
         <v>280.01</v>
       </c>
     </row>
-    <row r="6" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
+    <row r="6" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="12">
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="14">
         <f>SUM(D5)</f>
         <v>11.2004</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="11">
+      <c r="E6" s="15">
         <f>SUM(E5)</f>
         <v>280.01</v>
       </c>
     </row>
-    <row r="8" ht="32" customHeight="1" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+    <row r="8" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-    </row>
-    <row r="9" ht="32" customHeight="1" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="14" t="s">
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+    </row>
+    <row r="9" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-    </row>
-    <row r="10" ht="32" customHeight="1" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="14" t="s">
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+    </row>
+    <row r="10" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-    </row>
-    <row r="11" ht="32" customHeight="1" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+    </row>
+    <row r="11" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+    </row>
+    <row r="12" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A8:E8"/>
     <mergeCell ref="A9:E9"/>
     <mergeCell ref="A10:E10"/>
     <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A12:E12"/>
   </mergeCells>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
@@ -1020,7 +1079,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1030,7 +1089,7 @@
     <col min="5" max="5" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1049,33 +1108,33 @@
     </row>
     <row r="2" ht="25" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D2" s="6">
-        <v>8</v>
+        <v>2.0004</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" ht="25" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>7</v>
       </c>
       <c r="D3" s="6">
-        <v>1.2</v>
+        <v>8</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>8</v>
@@ -1083,27 +1142,27 @@
     </row>
     <row r="4" ht="25" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D4" s="6">
-        <v>2.0004</v>
+        <v>1.2</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>13</v>
@@ -1117,63 +1176,73 @@
         <v>280.01</v>
       </c>
     </row>
-    <row r="6" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
+    <row r="6" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="12">
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="14">
         <f>SUM(D5)</f>
         <v>11.2004</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="11">
+      <c r="E6" s="15">
         <f>SUM(E5)</f>
         <v>280.01</v>
       </c>
     </row>
-    <row r="8" ht="32" customHeight="1" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+    <row r="8" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-    </row>
-    <row r="9" ht="32" customHeight="1" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="14" t="s">
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+    </row>
+    <row r="9" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-    </row>
-    <row r="10" ht="32" customHeight="1" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="14" t="s">
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+    </row>
+    <row r="10" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-    </row>
-    <row r="11" ht="32" customHeight="1" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+    </row>
+    <row r="11" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+    </row>
+    <row r="12" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A8:E8"/>
     <mergeCell ref="A9:E9"/>
     <mergeCell ref="A10:E10"/>
     <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A12:E12"/>
   </mergeCells>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
@@ -1184,7 +1253,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1194,7 +1263,7 @@
     <col min="5" max="5" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1213,27 +1282,27 @@
     </row>
     <row r="2" ht="25" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D2" s="6">
         <v>8</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" ht="25" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>11</v>
@@ -1247,27 +1316,27 @@
     </row>
     <row r="4" ht="25" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D4" s="6">
         <v>1.2</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>13</v>
@@ -1281,63 +1350,73 @@
         <v>280.01</v>
       </c>
     </row>
-    <row r="6" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
+    <row r="6" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="12">
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="14">
         <f>SUM(D5)</f>
         <v>11.2004</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="11">
+      <c r="E6" s="15">
         <f>SUM(E5)</f>
         <v>280.01</v>
       </c>
     </row>
-    <row r="8" ht="32" customHeight="1" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+    <row r="8" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-    </row>
-    <row r="9" ht="32" customHeight="1" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="14" t="s">
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+    </row>
+    <row r="9" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-    </row>
-    <row r="10" ht="32" customHeight="1" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="14" t="s">
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+    </row>
+    <row r="10" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-    </row>
-    <row r="11" ht="32" customHeight="1" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+    </row>
+    <row r="11" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+    </row>
+    <row r="12" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A8:E8"/>
     <mergeCell ref="A9:E9"/>
     <mergeCell ref="A10:E10"/>
     <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A12:E12"/>
   </mergeCells>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Show empty version differences and package handover guide with fictional sample
</commit_message>
<xml_diff>
--- a/docs/虚构数据_2026-09_v1.xlsx
+++ b/docs/虚构数据_2026-09_v1.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="67">
   <si>
     <t>姓名</t>
   </si>
@@ -39,40 +39,61 @@
     <t>备注</t>
   </si>
   <si>
-    <t>林星禾</t>
+    <t>沈知遥</t>
   </si>
   <si>
     <t>0000001001</t>
   </si>
   <si>
-    <t>活动文案整理</t>
-  </si>
-  <si>
-    <t>真实工作8小时（虚构示例）</t>
-  </si>
-  <si>
-    <t>物料费用折算</t>
+    <t>迎新报道撰写</t>
+  </si>
+  <si>
+    <t>虚构示例：工作工时</t>
+  </si>
+  <si>
+    <t>宣传物料费用折算</t>
   </si>
   <si>
     <t>物料费30元÷25=1.2小时</t>
   </si>
   <si>
-    <t>交通费用折算</t>
-  </si>
-  <si>
-    <t>车费50.01元÷25=2.0004小时</t>
+    <t>活动交通费用折算</t>
+  </si>
+  <si>
+    <t>车费50元÷25=2小时，不另加金额</t>
   </si>
   <si>
     <t>个人合计</t>
   </si>
   <si>
+    <t>林星澄</t>
+  </si>
+  <si>
+    <t>0000001002</t>
+  </si>
+  <si>
+    <t>稿件校对与排版</t>
+  </si>
+  <si>
+    <t>虚构示例：含两轮校对</t>
+  </si>
+  <si>
+    <t>0000001010</t>
+  </si>
+  <si>
+    <t>活动快讯编辑</t>
+  </si>
+  <si>
+    <t>与0000001001同名但非同一人，按学号区分</t>
+  </si>
+  <si>
     <t>本组合计</t>
   </si>
   <si>
     <t>统计月份：2026-09 ｜ 导出时间：2026/9/30 18:00:00（北京时间） ｜ 版本：v1</t>
   </si>
   <si>
-    <t>已通过3条，11.2004小时，280.01元；合计行E列展示金额，明细E列为备注。</t>
+    <t>已通过5条，17.7小时，442.50元；合计行E列展示金额，明细E列为备注。</t>
   </si>
   <si>
     <t>费用已包含在工时内，不重复加款。正式记录排除0条；另有未提交草稿0条（仅数量）。</t>
@@ -84,16 +105,124 @@
     <t>已通过、已导出仅表示审核与整理进度，不代表款项已到账。</t>
   </si>
   <si>
+    <t>许沐川</t>
+  </si>
+  <si>
+    <t>0000001003</t>
+  </si>
+  <si>
+    <t>海报适配与输出</t>
+  </si>
+  <si>
+    <t>同一学生多条记录</t>
+  </si>
+  <si>
+    <t>活动海报设计</t>
+  </si>
+  <si>
+    <t>虚构示例：海报设计与修改</t>
+  </si>
+  <si>
     <t>陈知夏</t>
   </si>
   <si>
-    <t>0000001003</t>
-  </si>
-  <si>
     <t>0000001004</t>
   </si>
   <si>
+    <t>长图制作</t>
+  </si>
+  <si>
+    <t>含主视觉、标题与中文说明排版</t>
+  </si>
+  <si>
+    <t>已通过3条，10.75小时，268.75元；合计行E列展示金额，明细E列为备注。</t>
+  </si>
+  <si>
+    <t>跨组推文文案整理</t>
+  </si>
+  <si>
+    <t>同一学生跨组，保留文案组归属</t>
+  </si>
+  <si>
+    <t>唐时安</t>
+  </si>
+  <si>
     <t>0000001005</t>
+  </si>
+  <si>
+    <t>奖励工时示例</t>
+  </si>
+  <si>
+    <t>仅演示登记方式，不代表部门奖励标准</t>
+  </si>
+  <si>
+    <t>人物采访提纲整理</t>
+  </si>
+  <si>
+    <t>虚构示例：采访准备</t>
+  </si>
+  <si>
+    <t>已通过3条，7.5小时，187.50元；合计行E列展示金额，明细E列为备注。</t>
+  </si>
+  <si>
+    <t>宋念初</t>
+  </si>
+  <si>
+    <t>0000001006</t>
+  </si>
+  <si>
+    <t>活动车费折算</t>
+  </si>
+  <si>
+    <t>车费50.01元÷25=2.0004小时，禁止截断</t>
+  </si>
+  <si>
+    <t>联络物料费用折算</t>
+  </si>
+  <si>
+    <t>物料费30元÷25=1.2小时，费用不重复加算</t>
+  </si>
+  <si>
+    <t>季南枝</t>
+  </si>
+  <si>
+    <t>0000001007</t>
+  </si>
+  <si>
+    <t>嘉宾联络与现场协调</t>
+  </si>
+  <si>
+    <t>虚构示例：会前确认与会中协调</t>
+  </si>
+  <si>
+    <t>已通过3条，6.2004小时，155.01元；合计行E列展示金额，明细E列为备注。</t>
+  </si>
+  <si>
+    <t>顾书言</t>
+  </si>
+  <si>
+    <t>0000001008</t>
+  </si>
+  <si>
+    <t>组内管理与协调示例</t>
+  </si>
+  <si>
+    <t>虚构管理工时，仅演示维护方式，标准待部门确认</t>
+  </si>
+  <si>
+    <t>温以棠</t>
+  </si>
+  <si>
+    <t>0000001009</t>
+  </si>
+  <si>
+    <t>活动短片剪辑</t>
+  </si>
+  <si>
+    <t>虚构示例：完成剪辑与字幕校对</t>
+  </si>
+  <si>
+    <t>已通过2条，8.5小时，212.50元；合计行E列展示金额，明细E列为备注。</t>
   </si>
 </sst>
 </file>
@@ -557,7 +686,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -629,7 +758,7 @@
         <v>11</v>
       </c>
       <c r="D4" s="6">
-        <v>2.0004</v>
+        <v>2</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>12</v>
@@ -647,80 +776,152 @@
       </c>
       <c r="D5" s="10">
         <f>SUM(D2:D4)</f>
-        <v>11.2004</v>
+        <v>11.2</v>
       </c>
       <c r="E5" s="11">
         <f>ROUND(D5*25,2)</f>
-        <v>280.01</v>
-      </c>
-    </row>
-    <row r="6" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="6" ht="25" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="14">
-        <f>SUM(D5)</f>
-        <v>11.2004</v>
-      </c>
-      <c r="E6" s="15">
-        <f>SUM(E5)</f>
-        <v>280.01</v>
-      </c>
-    </row>
-    <row r="8" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="6">
+        <v>5.5</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="10">
+        <f>SUM(D6:D6)</f>
+        <v>5.5</v>
+      </c>
+      <c r="E7" s="11">
+        <f>ROUND(D7*25,2)</f>
+        <v>137.5</v>
+      </c>
+    </row>
+    <row r="8" ht="43" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-    </row>
-    <row r="9" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-    </row>
-    <row r="10" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-    </row>
-    <row r="11" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
+      <c r="C8" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="6">
+        <v>1</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="10">
+        <f>SUM(D8:D8)</f>
+        <v>1</v>
+      </c>
+      <c r="E9" s="11">
+        <f>ROUND(D9*25,2)</f>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="14">
+        <f>SUM(D5,D7,D9)</f>
+        <v>17.7</v>
+      </c>
+      <c r="E10" s="15">
+        <f>SUM(E5,E7,E9)</f>
+        <v>442.5</v>
+      </c>
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
     </row>
+    <row r="13" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+    </row>
+    <row r="14" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+    </row>
+    <row r="15" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+    </row>
+    <row r="16" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+    </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A8:E8"/>
-    <mergeCell ref="A9:E9"/>
-    <mergeCell ref="A10:E10"/>
-    <mergeCell ref="A11:E11"/>
     <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A16:E16"/>
   </mergeCells>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
@@ -731,7 +932,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -760,101 +961,111 @@
     </row>
     <row r="2" ht="25" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="D2" s="6">
-        <v>1.2</v>
+        <v>0.5</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" ht="25" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="D3" s="6">
-        <v>8</v>
+        <v>6.25</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" ht="25" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="6">
-        <v>2.0004</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="10">
-        <f>SUM(D2:D4)</f>
-        <v>11.2004</v>
-      </c>
-      <c r="E5" s="11">
-        <f>ROUND(D5*25,2)</f>
-        <v>280.01</v>
+      <c r="D4" s="10">
+        <f>SUM(D2:D3)</f>
+        <v>6.75</v>
+      </c>
+      <c r="E4" s="11">
+        <f>ROUND(D4*25,2)</f>
+        <v>168.75</v>
+      </c>
+    </row>
+    <row r="5" ht="25" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" s="6">
+        <v>4</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="6" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="14">
-        <f>SUM(D5)</f>
-        <v>11.2004</v>
-      </c>
-      <c r="E6" s="15">
-        <f>SUM(E5)</f>
-        <v>280.01</v>
-      </c>
-    </row>
-    <row r="8" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
+      <c r="A6" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="10">
+        <f>SUM(D5:D5)</f>
+        <v>4</v>
+      </c>
+      <c r="E6" s="11">
+        <f>ROUND(D6*25,2)</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="14">
+        <f>SUM(D4,D6)</f>
+        <v>10.75</v>
+      </c>
+      <c r="E7" s="15">
+        <f>SUM(E4,E6)</f>
+        <v>268.75</v>
+      </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -863,7 +1074,7 @@
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -872,7 +1083,7 @@
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -881,20 +1092,29 @@
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
     </row>
+    <row r="13" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+    </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A8:E8"/>
     <mergeCell ref="A9:E9"/>
     <mergeCell ref="A10:E10"/>
     <mergeCell ref="A11:E11"/>
     <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A13:E13"/>
   </mergeCells>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
@@ -905,7 +1125,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -934,101 +1154,111 @@
     </row>
     <row r="2" ht="25" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="6">
+        <v>2.5</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="10">
+        <f>SUM(D2:D2)</f>
+        <v>2.5</v>
+      </c>
+      <c r="E3" s="11">
+        <f>ROUND(D3*25,2)</f>
+        <v>62.5</v>
+      </c>
+    </row>
+    <row r="4" ht="43" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D4" s="6">
+        <v>1.5</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" ht="25" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="6">
+        <v>3.5</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="10">
+        <f>SUM(D4:D5)</f>
+        <v>5</v>
+      </c>
+      <c r="E6" s="11">
+        <f>ROUND(D6*25,2)</f>
+        <v>125</v>
+      </c>
+    </row>
+    <row r="7" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="6">
-        <v>8</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" ht="25" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="6">
-        <v>2.0004</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" ht="25" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="6">
-        <v>1.2</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="10">
-        <f>SUM(D2:D4)</f>
-        <v>11.2004</v>
-      </c>
-      <c r="E5" s="11">
-        <f>ROUND(D5*25,2)</f>
-        <v>280.01</v>
-      </c>
-    </row>
-    <row r="6" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="14">
-        <f>SUM(D5)</f>
-        <v>11.2004</v>
-      </c>
-      <c r="E6" s="15">
-        <f>SUM(E5)</f>
-        <v>280.01</v>
-      </c>
-    </row>
-    <row r="8" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="14">
+        <f>SUM(D3,D6)</f>
+        <v>7.5</v>
+      </c>
+      <c r="E7" s="15">
+        <f>SUM(E3,E6)</f>
+        <v>187.5</v>
+      </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -1037,7 +1267,7 @@
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -1046,7 +1276,7 @@
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -1055,20 +1285,29 @@
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
     </row>
+    <row r="13" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+    </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A8:E8"/>
     <mergeCell ref="A9:E9"/>
     <mergeCell ref="A10:E10"/>
     <mergeCell ref="A11:E11"/>
     <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A13:E13"/>
   </mergeCells>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
@@ -1079,7 +1318,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1106,103 +1345,113 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" ht="25" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" ht="43" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>20</v>
+        <v>47</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="D2" s="6">
         <v>2.0004</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" ht="25" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" ht="43" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>20</v>
+        <v>47</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>7</v>
+        <v>51</v>
       </c>
       <c r="D3" s="6">
-        <v>8</v>
+        <v>1.2</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" ht="25" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="6">
-        <v>1.2</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="C5" s="8" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="10">
-        <f>SUM(D2:D4)</f>
-        <v>11.2004</v>
-      </c>
-      <c r="E5" s="11">
-        <f>ROUND(D5*25,2)</f>
-        <v>280.01</v>
+      <c r="D4" s="10">
+        <f>SUM(D2:D3)</f>
+        <v>3.2004</v>
+      </c>
+      <c r="E4" s="11">
+        <f>ROUND(D4*25,2)</f>
+        <v>80.01</v>
+      </c>
+    </row>
+    <row r="5" ht="25" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D5" s="6">
+        <v>3</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="6" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="14">
-        <f>SUM(D5)</f>
-        <v>11.2004</v>
-      </c>
-      <c r="E6" s="15">
-        <f>SUM(E5)</f>
-        <v>280.01</v>
-      </c>
-    </row>
-    <row r="8" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
+      <c r="A6" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="10">
+        <f>SUM(D5:D5)</f>
+        <v>3</v>
+      </c>
+      <c r="E6" s="11">
+        <f>ROUND(D6*25,2)</f>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="14">
+        <f>SUM(D4,D6)</f>
+        <v>6.2004</v>
+      </c>
+      <c r="E7" s="15">
+        <f>SUM(E4,E6)</f>
+        <v>155.01</v>
+      </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -1211,7 +1460,7 @@
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>17</v>
+        <v>57</v>
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -1220,7 +1469,7 @@
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -1229,20 +1478,29 @@
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
     </row>
+    <row r="13" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+    </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A8:E8"/>
     <mergeCell ref="A9:E9"/>
     <mergeCell ref="A10:E10"/>
     <mergeCell ref="A11:E11"/>
     <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A13:E13"/>
   </mergeCells>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
@@ -1280,94 +1538,96 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" ht="25" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" ht="43" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>20</v>
+        <v>58</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>23</v>
+        <v>59</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>7</v>
+        <v>60</v>
       </c>
       <c r="D2" s="6">
-        <v>8</v>
+        <v>6.5</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" ht="25" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="6">
-        <v>2.0004</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>12</v>
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="10">
+        <f>SUM(D2:D2)</f>
+        <v>6.5</v>
+      </c>
+      <c r="E3" s="11">
+        <f>ROUND(D3*25,2)</f>
+        <v>162.5</v>
       </c>
     </row>
     <row r="4" ht="25" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>20</v>
+        <v>62</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>23</v>
+        <v>63</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="D4" s="6">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>10</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>20</v>
+        <v>62</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>23</v>
+        <v>63</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>13</v>
       </c>
       <c r="D5" s="10">
-        <f>SUM(D2:D4)</f>
-        <v>11.2004</v>
+        <f>SUM(D4:D4)</f>
+        <v>2</v>
       </c>
       <c r="E5" s="11">
         <f>ROUND(D5*25,2)</f>
-        <v>280.01</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" ht="25" customHeight="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B6" s="13"/>
       <c r="C6" s="13"/>
       <c r="D6" s="14">
-        <f>SUM(D5)</f>
-        <v>11.2004</v>
+        <f>SUM(D3,D5)</f>
+        <v>8.5</v>
       </c>
       <c r="E6" s="15">
-        <f>SUM(E5)</f>
-        <v>280.01</v>
+        <f>SUM(E3,E5)</f>
+        <v>212.5</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
@@ -1376,7 +1636,7 @@
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>16</v>
+        <v>66</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -1385,7 +1645,7 @@
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -1394,7 +1654,7 @@
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -1403,7 +1663,7 @@
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>

</xml_diff>